<commit_message>
display skipped empty columns, display progress, and agent thinking
</commit_message>
<xml_diff>
--- a/Yazan Test.xlsx
+++ b/Yazan Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Documents\Precursive Browser Agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB56B266-6E97-4FD6-9058-1263CC72F54B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8D9EE9-920E-41EA-96F2-FAC6B5B95E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A912A27F-21DA-4F3D-BECF-679CE1E950F8}"/>
   </bookViews>
@@ -149,9 +149,6 @@
     <t>05/06</t>
   </si>
   <si>
-    <t>McKinsey -Â Value Finder - SAP</t>
-  </si>
-  <si>
     <t>Project Evolve</t>
   </si>
   <si>
@@ -164,9 +161,6 @@
     <t>03 - Workflow Design &amp; Build</t>
   </si>
   <si>
-    <t>NMC</t>
-  </si>
-  <si>
     <t>Project Pulse</t>
   </si>
   <si>
@@ -177,6 +171,12 @@
   </si>
   <si>
     <t>06 - UAT Execution</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
   </si>
 </sst>
 </file>
@@ -208,7 +208,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -246,6 +246,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -259,14 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -290,6 +289,19 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -652,553 +664,543 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="2" t="s">
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="2" t="s">
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="2" t="s">
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="2" t="s">
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
+      <c r="Z1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="AA1" s="3"/>
-      <c r="AB1" s="3"/>
-      <c r="AC1" s="3"/>
-      <c r="AD1" s="3"/>
-      <c r="AE1" s="2" t="s">
+      <c r="AA1" s="10"/>
+      <c r="AB1" s="10"/>
+      <c r="AC1" s="10"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AF1" s="3"/>
-      <c r="AG1" s="3"/>
-      <c r="AH1" s="3"/>
-      <c r="AI1" s="3"/>
-      <c r="AJ1" s="3"/>
-      <c r="AK1" s="3"/>
-      <c r="AL1" s="2" t="s">
+      <c r="AF1" s="10"/>
+      <c r="AG1" s="10"/>
+      <c r="AH1" s="10"/>
+      <c r="AI1" s="10"/>
+      <c r="AJ1" s="10"/>
+      <c r="AK1" s="10"/>
+      <c r="AL1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="AM1" s="3"/>
-      <c r="AN1" s="3"/>
-      <c r="AO1" s="3"/>
-      <c r="AP1" s="3"/>
-      <c r="AQ1" s="2" t="s">
+      <c r="AM1" s="10"/>
+      <c r="AN1" s="10"/>
+      <c r="AO1" s="10"/>
+      <c r="AP1" s="10"/>
+      <c r="AQ1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="AR1" s="3"/>
-      <c r="AS1" s="2" t="s">
+      <c r="AR1" s="10"/>
+      <c r="AS1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="AT1" s="3"/>
-      <c r="AU1" s="3"/>
-      <c r="AV1" s="3"/>
-      <c r="AW1" s="3"/>
+      <c r="AT1" s="10"/>
+      <c r="AU1" s="10"/>
+      <c r="AV1" s="10"/>
+      <c r="AW1" s="10"/>
     </row>
     <row r="2" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4" t="s">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4" t="s">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="Q3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="R3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="S3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="T3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="U3" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6">
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3">
         <v>2</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
     </row>
     <row r="5" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="10">
-        <v>0.75</v>
-      </c>
-      <c r="E5" s="10">
+      <c r="C5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7">
         <v>1</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="13">
         <v>3.5</v>
       </c>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9"/>
-      <c r="T5" s="9"/>
-      <c r="U5" s="9"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
     </row>
     <row r="6" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="7">
+      <c r="C6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+      <c r="F6" s="12">
+        <v>4</v>
+      </c>
+      <c r="G6" s="4">
+        <v>1</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="I6" s="3"/>
+      <c r="J6" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="K6" s="4">
+        <v>2</v>
+      </c>
+      <c r="L6" s="3"/>
+      <c r="M6" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3">
+        <v>1</v>
+      </c>
+      <c r="R6" s="3">
         <v>1.25</v>
       </c>
-      <c r="E6" s="7">
-        <v>1</v>
-      </c>
-      <c r="F6" s="6">
-        <v>4</v>
-      </c>
-      <c r="G6" s="7">
-        <v>1</v>
-      </c>
-      <c r="H6" s="7">
-        <v>0.75</v>
-      </c>
-      <c r="I6" s="6"/>
-      <c r="J6" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="K6" s="7">
-        <v>2</v>
-      </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="7">
-        <v>0.75</v>
-      </c>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6">
-        <v>1</v>
-      </c>
-      <c r="R6" s="6">
+      <c r="S6" s="4">
         <v>1.25</v>
       </c>
-      <c r="S6" s="7">
-        <v>1.25</v>
-      </c>
-      <c r="T6" s="7">
+      <c r="T6" s="4">
         <v>0.5</v>
       </c>
-      <c r="U6" s="6"/>
+      <c r="U6" s="3"/>
     </row>
     <row r="7" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9">
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6">
         <v>2.35</v>
       </c>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="9"/>
-      <c r="U7" s="9"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
     </row>
     <row r="8" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6">
+      <c r="A8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3">
         <v>1.5</v>
       </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
     </row>
     <row r="9" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="11">
+      <c r="A9" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="6">
+        <v>5</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="8">
         <v>0.75</v>
       </c>
-      <c r="E9" s="11">
+      <c r="I9" s="6"/>
+      <c r="J9" s="8">
+        <v>1</v>
+      </c>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="8">
+        <v>1</v>
+      </c>
+      <c r="N9" s="8">
         <v>0.5</v>
       </c>
-      <c r="F9" s="9">
-        <v>5</v>
-      </c>
-      <c r="G9" s="9"/>
-      <c r="H9" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="I9" s="9"/>
-      <c r="J9" s="11">
-        <v>1</v>
-      </c>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="11">
-        <v>1</v>
-      </c>
-      <c r="N9" s="11">
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="8">
+        <v>0.25</v>
+      </c>
+      <c r="R9" s="8">
         <v>0.5</v>
       </c>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="11">
+      <c r="S9" s="8">
         <v>0.25</v>
       </c>
-      <c r="R9" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="S9" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
     </row>
     <row r="10" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="A10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6">
+      <c r="C10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3">
         <v>0.5</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="7">
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="4">
         <v>0.75</v>
       </c>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="7">
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="4">
         <v>0.5</v>
       </c>
-      <c r="S10" s="6"/>
-      <c r="T10" s="7">
+      <c r="S10" s="3"/>
+      <c r="T10" s="4">
         <v>3</v>
       </c>
-      <c r="U10" s="7">
+      <c r="U10" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="10">
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7">
         <v>2.5</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="7">
         <v>1.75</v>
       </c>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="10">
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="7">
         <v>0.5</v>
       </c>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="10">
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="7">
         <v>0.75</v>
       </c>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="10">
+      <c r="P11" s="6"/>
+      <c r="Q11" s="7">
         <v>1</v>
       </c>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="10">
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="7">
         <v>5.25</v>
       </c>
-      <c r="U11" s="10">
+      <c r="U11" s="7">
         <v>5.75</v>
       </c>
     </row>
     <row r="12" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="A12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6">
+      <c r="B12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3">
         <v>0.25</v>
       </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="7">
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="4">
         <v>0.75</v>
       </c>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
+      <c r="U12" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="T1:Y1"/>
-    <mergeCell ref="Z1:AD1"/>
-    <mergeCell ref="AE1:AK1"/>
-    <mergeCell ref="AL1:AP1"/>
-    <mergeCell ref="AQ1:AR1"/>
     <mergeCell ref="AS1:AW1"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:B3"/>
@@ -1206,6 +1208,11 @@
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="I1:M1"/>
     <mergeCell ref="N1:S1"/>
+    <mergeCell ref="T1:Y1"/>
+    <mergeCell ref="Z1:AD1"/>
+    <mergeCell ref="AE1:AK1"/>
+    <mergeCell ref="AL1:AP1"/>
+    <mergeCell ref="AQ1:AR1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>